<commit_message>
updated with calendar view
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mdigital-my.sharepoint.com/personal/m269810_one_merckgroup_com/Documents/Documents/LegacyHomeDriveDocuments/EFSPI/Calendar/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mdigital-my.sharepoint.com/personal/m269810_one_merckgroup_com/Documents/Documents/LegacyHomeDriveDocuments/EFSPI/EFSPI_Events_Calendar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C09BA042-B4F9-4453-98FD-F1168A7B8ABD}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{476E3C07-12AD-4DBA-BB2C-2A0FBAC9665C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{3AD4CD51-029A-4D3E-BCE9-D3BABE131D5C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Title</t>
   </si>
@@ -87,13 +87,76 @@
   </si>
   <si>
     <t>Frankfurt</t>
+  </si>
+  <si>
+    <t>Event 1</t>
+  </si>
+  <si>
+    <t>Org1</t>
+  </si>
+  <si>
+    <t>Loc1</t>
+  </si>
+  <si>
+    <t>Event 2</t>
+  </si>
+  <si>
+    <t>Org2</t>
+  </si>
+  <si>
+    <t>Loc2</t>
+  </si>
+  <si>
+    <t>Event 3</t>
+  </si>
+  <si>
+    <t>Org3</t>
+  </si>
+  <si>
+    <t>Loc3</t>
+  </si>
+  <si>
+    <t>Event 4</t>
+  </si>
+  <si>
+    <t>Org4</t>
+  </si>
+  <si>
+    <t>Loc4</t>
+  </si>
+  <si>
+    <t>Event 5</t>
+  </si>
+  <si>
+    <t>Org5</t>
+  </si>
+  <si>
+    <t>Loc5</t>
+  </si>
+  <si>
+    <t>Event 6</t>
+  </si>
+  <si>
+    <t>Org6</t>
+  </si>
+  <si>
+    <t>Loc6</t>
+  </si>
+  <si>
+    <t>Event 7</t>
+  </si>
+  <si>
+    <t>Org7</t>
+  </si>
+  <si>
+    <t>Loc7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +168,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -470,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7FF786E-2CBC-43F4-BB59-B074A7E1A64E}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -546,7 +615,106 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="1">
+        <v>46275</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="1">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="1">
+        <v>46278</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="1">
+        <v>46278</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{08031FF3-74EB-475B-9054-179DC0537DEE}"/>
     <hyperlink ref="H2" r:id="rId2" xr:uid="{E66C02CA-D8E7-4519-8470-B2567693CE50}"/>

</xml_diff>

<commit_message>
updated with new events
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mdigital-my.sharepoint.com/personal/m269810_one_merckgroup_com/Documents/Documents/LegacyHomeDriveDocuments/EFSPI/EFSPI_Events_Calendar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{476E3C07-12AD-4DBA-BB2C-2A0FBAC9665C}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A870E6D3-E6F9-4AF8-8F6D-84F6135D6012}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{3AD4CD51-029A-4D3E-BCE9-D3BABE131D5C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AD4CD51-029A-4D3E-BCE9-D3BABE131D5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Title</t>
   </si>
@@ -89,67 +89,73 @@
     <t>Frankfurt</t>
   </si>
   <si>
-    <t>Event 1</t>
-  </si>
-  <si>
-    <t>Org1</t>
-  </si>
-  <si>
-    <t>Loc1</t>
-  </si>
-  <si>
-    <t>Event 2</t>
-  </si>
-  <si>
-    <t>Org2</t>
-  </si>
-  <si>
-    <t>Loc2</t>
-  </si>
-  <si>
-    <t>Event 3</t>
-  </si>
-  <si>
-    <t>Org3</t>
-  </si>
-  <si>
-    <t>Loc3</t>
-  </si>
-  <si>
-    <t>Event 4</t>
-  </si>
-  <si>
-    <t>Org4</t>
-  </si>
-  <si>
-    <t>Loc4</t>
-  </si>
-  <si>
-    <t>Event 5</t>
-  </si>
-  <si>
-    <t>Org5</t>
-  </si>
-  <si>
-    <t>Loc5</t>
-  </si>
-  <si>
-    <t>Event 6</t>
-  </si>
-  <si>
-    <t>Org6</t>
-  </si>
-  <si>
-    <t>Loc6</t>
-  </si>
-  <si>
-    <t>Event 7</t>
-  </si>
-  <si>
-    <t>Org7</t>
-  </si>
-  <si>
-    <t>Loc7</t>
+    <t>Making Estimands Work - Practical Approaches with Implementation in Data Standards</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>online</t>
+  </si>
+  <si>
+    <t>15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>https://www.psiweb.org/events/event-item/2026/09/29/default-calendar/making-estimands-work---practical-approaches-with-implementation-in-data-standards__;!!Eu8ikxSnpXkBCg!ZnYE-4MUU38ZFe_chBltUeCgJdPd--goUozx1WuyBb1D4DlcqTXJ4Sy6slEdzy6hXQm02Gc2l-YIGMWHgOk6dEaZqAbaOb8753hrBzM$</t>
+  </si>
+  <si>
+    <t>Training Course: Adaptive Designs</t>
+  </si>
+  <si>
+    <t>GBP 310</t>
+  </si>
+  <si>
+    <t>free</t>
+  </si>
+  <si>
+    <t>free for members</t>
+  </si>
+  <si>
+    <t>EUR 300</t>
+  </si>
+  <si>
+    <t>https://www.psiweb.org/events/event-item/2026/10/20/default-calendar/psi-training-course--adaptive-designs__;!!Eu8ikxSnpXkBCg!ZnYE-4MUU38ZFe_chBltUeCgJdPd--goUozx1WuyBb1D4DlcqTXJ4Sy6slEdzy6hXQm02Gc2l-YIGMWHgOk6dEaZqAbaOb871MA6efM$</t>
+  </si>
+  <si>
+    <t>IBIG Forum</t>
+  </si>
+  <si>
+    <t>IBIG</t>
+  </si>
+  <si>
+    <t>Rome</t>
+  </si>
+  <si>
+    <t>https://eventi.linecongress.com/FrontEnd/index.php?job=CAMBIO_LINGUA&amp;SYSTEM_LINGUA=en&amp;center=REGISTRAZIONE__;!!Eu8ikxSnpXkBCg!cJTNL3lwAKtZ7hWJ_s9ypHmPSdzuYnQo1s8SMgA1jEizMlxwiY4vSqfa9BjDc6ctfJDakOF1p_NlqCm38WljlmKPu0xXmwSCoRz6$</t>
+  </si>
+  <si>
+    <t>see registration link</t>
+  </si>
+  <si>
+    <t>15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>EUR 60 + VAT</t>
+  </si>
+  <si>
+    <t>https://www.simef.it/events/webinar-series-on-digital-innovation-in-healthcare-ai-data-and-emerging-technologies/__;!!Eu8ikxSnpXkBCg!cJTNL3lwAKtZ7hWJ_s9ypHmPSdzuYnQo1s8SMgA1jEizMlxwiY4vSqfa9BjDc6ctfJDakOF1p_NlqCm38WljlmKPu0xXm_95G_2I$</t>
+  </si>
+  <si>
+    <t>Digital Innovation in Healthcare (1): AI, Data and Emerging Technologies</t>
+  </si>
+  <si>
+    <t>17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>Digital Innovation in Healthcare (2): AI, Data and Emerging Technologies</t>
+  </si>
+  <si>
+    <t>Digital Innovation in Healthcare (3): AI, Data and Emerging Technologies</t>
   </si>
 </sst>
 </file>
@@ -540,16 +546,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7FF786E-2CBC-43F4-BB59-B074A7E1A64E}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -575,7 +581,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -588,8 +594,8 @@
       <c r="D2" s="1">
         <v>46253</v>
       </c>
-      <c r="F2">
-        <v>300</v>
+      <c r="F2" t="s">
+        <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
@@ -598,7 +604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -611,11 +617,11 @@
       <c r="D3" s="1">
         <v>46353</v>
       </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -626,98 +632,141 @@
         <v>18</v>
       </c>
       <c r="D4" s="1">
-        <v>46260</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46294</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D5" s="1">
-        <v>46266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46315</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1">
-        <v>46266</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46317</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1">
-        <v>46275</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46279</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1">
-        <v>46277</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46345</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1">
+        <v>46370</v>
+      </c>
+      <c r="E9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="F9" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="1">
-        <v>46278</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="H9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="1">
-        <v>46278</v>
-      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D10" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{08031FF3-74EB-475B-9054-179DC0537DEE}"/>
     <hyperlink ref="H2" r:id="rId2" xr:uid="{E66C02CA-D8E7-4519-8470-B2567693CE50}"/>
+    <hyperlink ref="H4" r:id="rId3" display="https://www.psiweb.org/events/event-item/2026/09/29/default-calendar/making-estimands-work---practical-approaches-with-implementation-in-data-standards__;!!Eu8ikxSnpXkBCg!ZnYE-4MUU38ZFe_chBltUeCgJdPd--goUozx1WuyBb1D4DlcqTXJ4Sy6slEdzy6hXQm02Gc2l-YIGMWHgOk6dEaZqAbaOb8753hrBzM$" xr:uid="{47929054-A7F1-48F3-A09C-5F409B8DF899}"/>
+    <hyperlink ref="H5" r:id="rId4" xr:uid="{8F27C399-5F6E-4931-9754-F6027C6D2887}"/>
+    <hyperlink ref="H6" r:id="rId5" xr:uid="{5B6532C3-6300-4EF1-817B-5370743FBED2}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{74B81336-B77E-4FE3-B292-3EC638C8D38C}"/>
+    <hyperlink ref="H8" r:id="rId7" xr:uid="{89A74A77-045F-48B7-87C5-97737ACA562C}"/>
+    <hyperlink ref="H9" r:id="rId8" xr:uid="{9D96AAE2-3517-4194-AB05-F87AF4D3141C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>